<commit_message>
add more 4 test case for events (switch registration type from standard, switch registration type from group, remove player, keep player)
</commit_message>
<xml_diff>
--- a/data/test_data_swing_mobile.xlsx
+++ b/data/test_data_swing_mobile.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="16360" tabRatio="500" activeTab="3"/>
+    <workbookView windowHeight="17160" tabRatio="500" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Driving_Range" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="147">
   <si>
     <t>ACTION</t>
   </si>
@@ -401,6 +401,9 @@
     <t>REGISTRATION_TIME</t>
   </si>
   <si>
+    <t>SWITCH_REGISTRATION_TYPE</t>
+  </si>
+  <si>
     <t>TC_E_001</t>
   </si>
   <si>
@@ -441,6 +444,33 @@
   </si>
   <si>
     <t>Joko</t>
+  </si>
+  <si>
+    <t>TC_E_004</t>
+  </si>
+  <si>
+    <t>Swith from Standard to Group Registration Booking</t>
+  </si>
+  <si>
+    <t>Tournament AIGG Test</t>
+  </si>
+  <si>
+    <t>TC_E_005</t>
+  </si>
+  <si>
+    <t>Swith from Group to Standard Registration Booking</t>
+  </si>
+  <si>
+    <t>TC_E_006</t>
+  </si>
+  <si>
+    <t>Keep player case</t>
+  </si>
+  <si>
+    <t>TC_E_007</t>
+  </si>
+  <si>
+    <t>Remove player case</t>
   </si>
 </sst>
 </file>
@@ -2355,19 +2385,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="7"/>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="14.4" outlineLevelRow="7"/>
   <cols>
     <col min="2" max="2" width="12.1964285714286" customWidth="1"/>
-    <col min="3" max="3" width="26.1875" customWidth="1"/>
+    <col min="3" max="3" width="48.0625" customWidth="1"/>
     <col min="4" max="4" width="28.125" customWidth="1"/>
     <col min="5" max="5" width="19.7857142857143" customWidth="1"/>
     <col min="6" max="6" width="20.2321428571429" customWidth="1"/>
     <col min="7" max="7" width="29.0178571428571" customWidth="1"/>
     <col min="8" max="8" width="20.3839285714286" customWidth="1"/>
+    <col min="9" max="9" width="30.9285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" spans="1:8">
+    <row r="1" ht="15" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2392,74 +2423,181 @@
       <c r="H1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H4" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E5" t="s">
+        <v>131</v>
+      </c>
+      <c r="F5" t="s">
+        <v>132</v>
+      </c>
+      <c r="G5" t="s">
+        <v>133</v>
+      </c>
+      <c r="H5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D6" t="s">
+        <v>140</v>
+      </c>
+      <c r="E6" t="s">
+        <v>136</v>
+      </c>
+      <c r="F6" t="s">
+        <v>132</v>
+      </c>
+      <c r="G6" t="s">
+        <v>133</v>
+      </c>
+      <c r="H6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7" t="s">
+        <v>131</v>
+      </c>
+      <c r="F7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E8" t="s">
+        <v>131</v>
+      </c>
+      <c r="F8" t="s">
+        <v>132</v>
+      </c>
+      <c r="G8" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add 8 multisports testcase
</commit_message>
<xml_diff>
--- a/data/test_data_swing_mobile.xlsx
+++ b/data/test_data_swing_mobile.xlsx
@@ -4,13 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17160" tabRatio="500" activeTab="3"/>
+    <workbookView windowHeight="17160" tabRatio="500" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Driving_Range" sheetId="1" r:id="rId1"/>
     <sheet name="Tee_Time" sheetId="2" r:id="rId2"/>
     <sheet name="Tee_Time_Player" sheetId="3" r:id="rId3"/>
     <sheet name="Events" sheetId="4" r:id="rId4"/>
+    <sheet name="Multisport" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="170">
   <si>
     <t>ACTION</t>
   </si>
@@ -471,6 +472,75 @@
   </si>
   <si>
     <t>Remove player case</t>
+  </si>
+  <si>
+    <t>SPORT_NAME</t>
+  </si>
+  <si>
+    <t>VENUE_NAME</t>
+  </si>
+  <si>
+    <t>TITLE_SCHEDULE</t>
+  </si>
+  <si>
+    <t>HOW_MUCH_SCHEDULE</t>
+  </si>
+  <si>
+    <t>TC_MLTS_001</t>
+  </si>
+  <si>
+    <t>Verify user can choose sport from sport option page</t>
+  </si>
+  <si>
+    <t>BILLIARD</t>
+  </si>
+  <si>
+    <t>TC_MLTS_002</t>
+  </si>
+  <si>
+    <t>Verify user can choose venue</t>
+  </si>
+  <si>
+    <t>BillWithPPD</t>
+  </si>
+  <si>
+    <t>TC_MLTS_003</t>
+  </si>
+  <si>
+    <t>Verify user can book venue</t>
+  </si>
+  <si>
+    <t>TC_MLTS_004</t>
+  </si>
+  <si>
+    <t>Verify user can select schedule</t>
+  </si>
+  <si>
+    <t>table1</t>
+  </si>
+  <si>
+    <t>TC_MLTS_005</t>
+  </si>
+  <si>
+    <t>Verify user can select add player</t>
+  </si>
+  <si>
+    <t>TC_MLTS_006</t>
+  </si>
+  <si>
+    <t>Verify user can remove player</t>
+  </si>
+  <si>
+    <t>TC_MLTS_007</t>
+  </si>
+  <si>
+    <t>Verify user can select payment</t>
+  </si>
+  <si>
+    <t>TC_MLTS_008</t>
+  </si>
+  <si>
+    <t>Verify user can book venue end to end until payment</t>
   </si>
 </sst>
 </file>
@@ -2604,4 +2674,205 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultColWidth="30.2053571428571" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <cols>
+    <col min="1" max="1" width="30.2053571428571" customWidth="1"/>
+    <col min="2" max="2" width="45.375" customWidth="1"/>
+    <col min="3" max="3" width="41.0714285714286" customWidth="1"/>
+    <col min="4" max="16384" width="30.2053571428571" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F1" t="s">
+        <v>150</v>
+      </c>
+      <c r="G1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B4" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" t="s">
+        <v>156</v>
+      </c>
+      <c r="E5" t="s">
+        <v>161</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" customFormat="1" spans="1:8">
+      <c r="A6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" t="s">
+        <v>156</v>
+      </c>
+      <c r="E6" t="s">
+        <v>161</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" t="s">
+        <v>165</v>
+      </c>
+      <c r="C7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D7" t="s">
+        <v>156</v>
+      </c>
+      <c r="E7" t="s">
+        <v>161</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B8" t="s">
+        <v>167</v>
+      </c>
+      <c r="C8" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" t="s">
+        <v>156</v>
+      </c>
+      <c r="E8" t="s">
+        <v>161</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>168</v>
+      </c>
+      <c r="B9" t="s">
+        <v>169</v>
+      </c>
+      <c r="C9" t="s">
+        <v>153</v>
+      </c>
+      <c r="D9" t="s">
+        <v>156</v>
+      </c>
+      <c r="E9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9" t="s">
+        <v>137</v>
+      </c>
+      <c r="H9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>